<commit_message>
Add support for BP (Base Pointer) register in parse_reg function
</commit_message>
<xml_diff>
--- a/LEAF ISA.xlsx
+++ b/LEAF ISA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kyhyh\Desktop\LEAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA880C6D-5273-4E9B-85F4-44F1E57A344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE071C8-3588-441C-B198-8E8634DE53C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="406" xr2:uid="{8647DCE3-3E5E-4484-B9D8-47B9DC77BDB4}"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" tabRatio="406" xr2:uid="{8647DCE3-3E5E-4484-B9D8-47B9DC77BDB4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,7 +125,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K47" authorId="0" shapeId="0" xr:uid="{301BB7AB-65B7-49F1-8BC0-4E9BA1485772}">
+    <comment ref="K45" authorId="0" shapeId="0" xr:uid="{301BB7AB-65B7-49F1-8BC0-4E9BA1485772}">
       <text>
         <r>
           <rPr>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="143">
   <si>
     <t>Instruction</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -452,14 +452,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PSH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>POP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CMP</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -469,16 +461,6 @@
   </si>
   <si>
     <t>SUB R0, src1,  src2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>dest = MEM[SP]
-SP = SP + offset</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MEM[SP + offset] = src
-SP = SP + offset</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -663,10 +645,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>sign-extended offset</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>R1 - R14</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -743,6 +721,15 @@
   <si>
     <t>PC = call address
 push PC + 1 into return address stack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>R14
+(BP)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>base pointer register</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -786,7 +773,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -799,14 +786,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1135,13 +1116,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1199,98 +1206,101 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1626,7 +1636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4394A859-953B-40A0-A8C8-6ED823E9FBE3}">
-  <dimension ref="A1:AQ48"/>
+  <dimension ref="A1:AQ46"/>
   <sheetFormatPr defaultRowHeight="18.600000000000001" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.59765625" style="2" customWidth="1"/>
@@ -1641,97 +1651,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="58.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="36"/>
-      <c r="V1" s="36"/>
-      <c r="W1" s="36"/>
-      <c r="X1" s="36"/>
-      <c r="Y1" s="36"/>
-      <c r="Z1" s="36"/>
-      <c r="AA1" s="36"/>
-      <c r="AB1" s="36"/>
-      <c r="AC1" s="36"/>
-      <c r="AD1" s="36"/>
-      <c r="AE1" s="36"/>
-      <c r="AF1" s="36"/>
-      <c r="AG1" s="36"/>
-      <c r="AH1" s="36"/>
-      <c r="AI1" s="36"/>
-      <c r="AJ1" s="36"/>
-      <c r="AK1" s="36"/>
-      <c r="AL1" s="37"/>
+      <c r="A1" s="45" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="46"/>
+      <c r="AA1" s="46"/>
+      <c r="AB1" s="46"/>
+      <c r="AC1" s="46"/>
+      <c r="AD1" s="46"/>
+      <c r="AE1" s="46"/>
+      <c r="AF1" s="46"/>
+      <c r="AG1" s="46"/>
+      <c r="AH1" s="46"/>
+      <c r="AI1" s="46"/>
+      <c r="AJ1" s="46"/>
+      <c r="AK1" s="46"/>
+      <c r="AL1" s="47"/>
     </row>
     <row r="2" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="41" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42" t="s">
+      <c r="A2" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42" t="s">
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="34"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="42"/>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42" t="s">
+      <c r="T2" s="34"/>
+      <c r="U2" s="34"/>
+      <c r="V2" s="34"/>
+      <c r="W2" s="34"/>
+      <c r="X2" s="34"/>
+      <c r="Y2" s="34"/>
+      <c r="Z2" s="34"/>
+      <c r="AA2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="AB2" s="42"/>
-      <c r="AC2" s="42"/>
-      <c r="AD2" s="42"/>
-      <c r="AE2" s="42"/>
-      <c r="AF2" s="42"/>
-      <c r="AG2" s="42"/>
-      <c r="AH2" s="40"/>
-      <c r="AJ2" s="39" t="s">
+      <c r="AB2" s="34"/>
+      <c r="AC2" s="34"/>
+      <c r="AD2" s="34"/>
+      <c r="AE2" s="34"/>
+      <c r="AF2" s="34"/>
+      <c r="AG2" s="34"/>
+      <c r="AH2" s="31"/>
+      <c r="AJ2" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="AK2" s="42"/>
-      <c r="AL2" s="40" t="s">
+      <c r="AK2" s="34"/>
+      <c r="AL2" s="31" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1742,53 +1752,53 @@
       <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="46" t="s">
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="43"/>
-      <c r="K3" s="44" t="s">
+      <c r="J3" s="36"/>
+      <c r="K3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="44"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="44"/>
-      <c r="W3" s="44"/>
-      <c r="X3" s="44"/>
-      <c r="Y3" s="44"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="44"/>
-      <c r="AB3" s="44"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="44"/>
-      <c r="AE3" s="44"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="44"/>
-      <c r="AH3" s="45"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="37"/>
+      <c r="W3" s="37"/>
+      <c r="X3" s="37"/>
+      <c r="Y3" s="37"/>
+      <c r="Z3" s="37"/>
+      <c r="AA3" s="37"/>
+      <c r="AB3" s="37"/>
+      <c r="AC3" s="37"/>
+      <c r="AD3" s="37"/>
+      <c r="AE3" s="37"/>
+      <c r="AF3" s="37"/>
+      <c r="AG3" s="37"/>
+      <c r="AH3" s="32"/>
       <c r="AJ3" s="7" t="s">
         <v>6</v>
       </c>
       <c r="AK3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AL3" s="45"/>
+      <c r="AL3" s="32"/>
     </row>
-    <row r="4" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="16" t="s">
         <v>9</v>
       </c>
@@ -1819,32 +1829,32 @@
       <c r="J4" s="15">
         <v>0</v>
       </c>
-      <c r="K4" s="47">
-        <v>0</v>
-      </c>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48"/>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="48"/>
-      <c r="S4" s="48"/>
-      <c r="T4" s="48"/>
-      <c r="U4" s="48"/>
-      <c r="V4" s="48"/>
-      <c r="W4" s="48"/>
-      <c r="X4" s="48"/>
-      <c r="Y4" s="48"/>
-      <c r="Z4" s="48"/>
-      <c r="AA4" s="48"/>
-      <c r="AB4" s="48"/>
-      <c r="AC4" s="48"/>
-      <c r="AD4" s="48"/>
-      <c r="AE4" s="48"/>
-      <c r="AF4" s="48"/>
-      <c r="AG4" s="48"/>
-      <c r="AH4" s="49"/>
+      <c r="K4" s="39">
+        <v>0</v>
+      </c>
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+      <c r="O4" s="40"/>
+      <c r="P4" s="40"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="40"/>
+      <c r="S4" s="40"/>
+      <c r="T4" s="40"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="40"/>
+      <c r="W4" s="40"/>
+      <c r="X4" s="40"/>
+      <c r="Y4" s="40"/>
+      <c r="Z4" s="40"/>
+      <c r="AA4" s="40"/>
+      <c r="AB4" s="40"/>
+      <c r="AC4" s="40"/>
+      <c r="AD4" s="40"/>
+      <c r="AE4" s="40"/>
+      <c r="AF4" s="40"/>
+      <c r="AG4" s="40"/>
+      <c r="AH4" s="41"/>
       <c r="AJ4" s="10" t="s">
         <v>27</v>
       </c>
@@ -1855,7 +1865,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
@@ -1886,38 +1896,38 @@
       <c r="J5" s="6">
         <v>0</v>
       </c>
-      <c r="K5" s="23" t="s">
+      <c r="K5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28" t="s">
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="28"/>
-      <c r="R5" s="28"/>
-      <c r="S5" s="28" t="s">
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="28"/>
-      <c r="W5" s="33">
-        <v>0</v>
-      </c>
-      <c r="X5" s="33"/>
-      <c r="Y5" s="33"/>
-      <c r="Z5" s="33"/>
-      <c r="AA5" s="33"/>
-      <c r="AB5" s="33"/>
-      <c r="AC5" s="33"/>
-      <c r="AD5" s="33"/>
-      <c r="AE5" s="33"/>
-      <c r="AF5" s="33"/>
-      <c r="AG5" s="33"/>
-      <c r="AH5" s="34"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="22">
+        <v>0</v>
+      </c>
+      <c r="X5" s="22"/>
+      <c r="Y5" s="22"/>
+      <c r="Z5" s="22"/>
+      <c r="AA5" s="22"/>
+      <c r="AB5" s="22"/>
+      <c r="AC5" s="22"/>
+      <c r="AD5" s="22"/>
+      <c r="AE5" s="22"/>
+      <c r="AF5" s="22"/>
+      <c r="AG5" s="22"/>
+      <c r="AH5" s="23"/>
       <c r="AJ5" s="5" t="s">
         <v>24</v>
       </c>
@@ -1928,7 +1938,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="5" t="s">
         <v>17</v>
       </c>
@@ -1959,38 +1969,38 @@
       <c r="J6" s="6">
         <v>0</v>
       </c>
-      <c r="K6" s="23" t="s">
+      <c r="K6" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28" t="s">
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28" t="s">
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T6" s="28"/>
-      <c r="U6" s="28"/>
-      <c r="V6" s="28"/>
-      <c r="W6" s="33">
-        <v>0</v>
-      </c>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="33"/>
-      <c r="AF6" s="33"/>
-      <c r="AG6" s="33"/>
-      <c r="AH6" s="34"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="22">
+        <v>0</v>
+      </c>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="22"/>
+      <c r="Z6" s="22"/>
+      <c r="AA6" s="22"/>
+      <c r="AB6" s="22"/>
+      <c r="AC6" s="22"/>
+      <c r="AD6" s="22"/>
+      <c r="AE6" s="22"/>
+      <c r="AF6" s="22"/>
+      <c r="AG6" s="22"/>
+      <c r="AH6" s="23"/>
       <c r="AJ6" s="5" t="s">
         <v>25</v>
       </c>
@@ -2001,7 +2011,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -2032,38 +2042,38 @@
       <c r="J7" s="6">
         <v>0</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L7" s="28"/>
-      <c r="M7" s="28"/>
-      <c r="N7" s="28"/>
-      <c r="O7" s="28" t="s">
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="28"/>
-      <c r="S7" s="28" t="s">
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="28"/>
-      <c r="U7" s="28"/>
-      <c r="V7" s="28"/>
-      <c r="W7" s="33">
-        <v>0</v>
-      </c>
-      <c r="X7" s="33"/>
-      <c r="Y7" s="33"/>
-      <c r="Z7" s="33"/>
-      <c r="AA7" s="33"/>
-      <c r="AB7" s="33"/>
-      <c r="AC7" s="33"/>
-      <c r="AD7" s="33"/>
-      <c r="AE7" s="33"/>
-      <c r="AF7" s="33"/>
-      <c r="AG7" s="33"/>
-      <c r="AH7" s="34"/>
+      <c r="T7" s="21"/>
+      <c r="U7" s="21"/>
+      <c r="V7" s="21"/>
+      <c r="W7" s="22">
+        <v>0</v>
+      </c>
+      <c r="X7" s="22"/>
+      <c r="Y7" s="22"/>
+      <c r="Z7" s="22"/>
+      <c r="AA7" s="22"/>
+      <c r="AB7" s="22"/>
+      <c r="AC7" s="22"/>
+      <c r="AD7" s="22"/>
+      <c r="AE7" s="22"/>
+      <c r="AF7" s="22"/>
+      <c r="AG7" s="22"/>
+      <c r="AH7" s="23"/>
       <c r="AJ7" s="5" t="s">
         <v>69</v>
       </c>
@@ -2074,7 +2084,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
@@ -2105,49 +2115,49 @@
       <c r="J8" s="6">
         <v>0</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="28"/>
-      <c r="M8" s="28"/>
-      <c r="N8" s="28"/>
-      <c r="O8" s="28" t="s">
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P8" s="28"/>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="28"/>
-      <c r="S8" s="28" t="s">
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T8" s="28"/>
-      <c r="U8" s="28"/>
-      <c r="V8" s="28"/>
-      <c r="W8" s="33">
-        <v>0</v>
-      </c>
-      <c r="X8" s="33"/>
-      <c r="Y8" s="33"/>
-      <c r="Z8" s="33"/>
-      <c r="AA8" s="33"/>
-      <c r="AB8" s="33"/>
-      <c r="AC8" s="33"/>
-      <c r="AD8" s="33"/>
-      <c r="AE8" s="33"/>
-      <c r="AF8" s="33"/>
-      <c r="AG8" s="33"/>
-      <c r="AH8" s="34"/>
+      <c r="T8" s="21"/>
+      <c r="U8" s="21"/>
+      <c r="V8" s="21"/>
+      <c r="W8" s="22">
+        <v>0</v>
+      </c>
+      <c r="X8" s="22"/>
+      <c r="Y8" s="22"/>
+      <c r="Z8" s="22"/>
+      <c r="AA8" s="22"/>
+      <c r="AB8" s="22"/>
+      <c r="AC8" s="22"/>
+      <c r="AD8" s="22"/>
+      <c r="AE8" s="22"/>
+      <c r="AF8" s="22"/>
+      <c r="AG8" s="22"/>
+      <c r="AH8" s="23"/>
       <c r="AJ8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="AL8" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="AK8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="AL8" s="6" t="s">
-        <v>78</v>
-      </c>
     </row>
-    <row r="9" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2178,49 +2188,49 @@
       <c r="J9" s="6">
         <v>0</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="28"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="28" t="s">
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
-      <c r="S9" s="28" t="s">
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T9" s="28"/>
-      <c r="U9" s="28"/>
-      <c r="V9" s="28"/>
-      <c r="W9" s="33">
-        <v>0</v>
-      </c>
-      <c r="X9" s="33"/>
-      <c r="Y9" s="33"/>
-      <c r="Z9" s="33"/>
-      <c r="AA9" s="33"/>
-      <c r="AB9" s="33"/>
-      <c r="AC9" s="33"/>
-      <c r="AD9" s="33"/>
-      <c r="AE9" s="33"/>
-      <c r="AF9" s="33"/>
-      <c r="AG9" s="33"/>
-      <c r="AH9" s="34"/>
+      <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
+      <c r="V9" s="21"/>
+      <c r="W9" s="22">
+        <v>0</v>
+      </c>
+      <c r="X9" s="22"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="22"/>
+      <c r="AA9" s="22"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="22"/>
+      <c r="AD9" s="22"/>
+      <c r="AE9" s="22"/>
+      <c r="AF9" s="22"/>
+      <c r="AG9" s="22"/>
+      <c r="AH9" s="23"/>
       <c r="AJ9" s="5" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AL9" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
@@ -2251,49 +2261,49 @@
       <c r="J10" s="6">
         <v>0</v>
       </c>
-      <c r="K10" s="23" t="s">
+      <c r="K10" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="28" t="s">
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P10" s="28"/>
-      <c r="Q10" s="28"/>
-      <c r="R10" s="28"/>
-      <c r="S10" s="28" t="s">
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T10" s="28"/>
-      <c r="U10" s="28"/>
-      <c r="V10" s="28"/>
-      <c r="W10" s="33">
-        <v>0</v>
-      </c>
-      <c r="X10" s="33"/>
-      <c r="Y10" s="33"/>
-      <c r="Z10" s="33"/>
-      <c r="AA10" s="33"/>
-      <c r="AB10" s="33"/>
-      <c r="AC10" s="33"/>
-      <c r="AD10" s="33"/>
-      <c r="AE10" s="33"/>
-      <c r="AF10" s="33"/>
-      <c r="AG10" s="33"/>
-      <c r="AH10" s="34"/>
+      <c r="T10" s="21"/>
+      <c r="U10" s="21"/>
+      <c r="V10" s="21"/>
+      <c r="W10" s="22">
+        <v>0</v>
+      </c>
+      <c r="X10" s="22"/>
+      <c r="Y10" s="22"/>
+      <c r="Z10" s="22"/>
+      <c r="AA10" s="22"/>
+      <c r="AB10" s="22"/>
+      <c r="AC10" s="22"/>
+      <c r="AD10" s="22"/>
+      <c r="AE10" s="22"/>
+      <c r="AF10" s="22"/>
+      <c r="AG10" s="22"/>
+      <c r="AH10" s="23"/>
       <c r="AJ10" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK10" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AL10" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="AK10" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="AL10" s="6" t="s">
-        <v>103</v>
-      </c>
     </row>
-    <row r="11" spans="1:38" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:38" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
@@ -2324,49 +2334,49 @@
       <c r="J11" s="6">
         <v>0</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="K11" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L11" s="28"/>
-      <c r="M11" s="28"/>
-      <c r="N11" s="28"/>
-      <c r="O11" s="28" t="s">
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="21"/>
+      <c r="O11" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P11" s="28"/>
-      <c r="Q11" s="28"/>
-      <c r="R11" s="28"/>
-      <c r="S11" s="28" t="s">
+      <c r="P11" s="21"/>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="21"/>
+      <c r="S11" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T11" s="28"/>
-      <c r="U11" s="28"/>
-      <c r="V11" s="28"/>
-      <c r="W11" s="33">
-        <v>0</v>
-      </c>
-      <c r="X11" s="33"/>
-      <c r="Y11" s="33"/>
-      <c r="Z11" s="33"/>
-      <c r="AA11" s="33"/>
-      <c r="AB11" s="33"/>
-      <c r="AC11" s="33"/>
-      <c r="AD11" s="33"/>
-      <c r="AE11" s="33"/>
-      <c r="AF11" s="33"/>
-      <c r="AG11" s="33"/>
-      <c r="AH11" s="34"/>
+      <c r="T11" s="21"/>
+      <c r="U11" s="21"/>
+      <c r="V11" s="21"/>
+      <c r="W11" s="22">
+        <v>0</v>
+      </c>
+      <c r="X11" s="22"/>
+      <c r="Y11" s="22"/>
+      <c r="Z11" s="22"/>
+      <c r="AA11" s="22"/>
+      <c r="AB11" s="22"/>
+      <c r="AC11" s="22"/>
+      <c r="AD11" s="22"/>
+      <c r="AE11" s="22"/>
+      <c r="AF11" s="22"/>
+      <c r="AG11" s="22"/>
+      <c r="AH11" s="23"/>
       <c r="AJ11" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="AK11" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="AL11" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="AK11" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="AL11" s="8" t="s">
-        <v>104</v>
-      </c>
     </row>
-    <row r="12" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="5" t="s">
         <v>23</v>
       </c>
@@ -2397,45 +2407,45 @@
       <c r="J12" s="6">
         <v>0</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="K12" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
-      <c r="O12" s="28" t="s">
+      <c r="L12" s="21"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P12" s="28"/>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="28"/>
-      <c r="S12" s="28" t="s">
+      <c r="P12" s="21"/>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="21"/>
+      <c r="S12" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T12" s="28"/>
-      <c r="U12" s="28"/>
-      <c r="V12" s="28"/>
-      <c r="W12" s="33">
-        <v>0</v>
-      </c>
-      <c r="X12" s="33"/>
-      <c r="Y12" s="33"/>
-      <c r="Z12" s="33"/>
-      <c r="AA12" s="33"/>
-      <c r="AB12" s="33"/>
-      <c r="AC12" s="33"/>
-      <c r="AD12" s="33"/>
-      <c r="AE12" s="33"/>
-      <c r="AF12" s="33"/>
-      <c r="AG12" s="33"/>
-      <c r="AH12" s="34"/>
+      <c r="T12" s="21"/>
+      <c r="U12" s="21"/>
+      <c r="V12" s="21"/>
+      <c r="W12" s="22">
+        <v>0</v>
+      </c>
+      <c r="X12" s="22"/>
+      <c r="Y12" s="22"/>
+      <c r="Z12" s="22"/>
+      <c r="AA12" s="22"/>
+      <c r="AB12" s="22"/>
+      <c r="AC12" s="22"/>
+      <c r="AD12" s="22"/>
+      <c r="AE12" s="22"/>
+      <c r="AF12" s="22"/>
+      <c r="AG12" s="22"/>
+      <c r="AH12" s="23"/>
     </row>
-    <row r="13" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -2461,43 +2471,43 @@
       <c r="J13" s="6">
         <v>0</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="K13" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="28"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="28"/>
-      <c r="O13" s="28" t="s">
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P13" s="28"/>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="28"/>
-      <c r="S13" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T13" s="28"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="28"/>
-      <c r="W13" s="28"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
-      <c r="Z13" s="28"/>
-      <c r="AA13" s="28"/>
-      <c r="AB13" s="28"/>
-      <c r="AC13" s="28"/>
-      <c r="AD13" s="28"/>
-      <c r="AE13" s="28"/>
-      <c r="AF13" s="28"/>
-      <c r="AG13" s="28"/>
-      <c r="AH13" s="29"/>
+      <c r="P13" s="21"/>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="21"/>
+      <c r="S13" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T13" s="21"/>
+      <c r="U13" s="21"/>
+      <c r="V13" s="21"/>
+      <c r="W13" s="21"/>
+      <c r="X13" s="21"/>
+      <c r="Y13" s="21"/>
+      <c r="Z13" s="21"/>
+      <c r="AA13" s="21"/>
+      <c r="AB13" s="21"/>
+      <c r="AC13" s="21"/>
+      <c r="AD13" s="21"/>
+      <c r="AE13" s="21"/>
+      <c r="AF13" s="21"/>
+      <c r="AG13" s="21"/>
+      <c r="AH13" s="30"/>
     </row>
-    <row r="14" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C14" s="5">
         <v>1</v>
@@ -2523,43 +2533,43 @@
       <c r="J14" s="6">
         <v>0</v>
       </c>
-      <c r="K14" s="23" t="s">
+      <c r="K14" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L14" s="28"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="28"/>
-      <c r="O14" s="28" t="s">
+      <c r="L14" s="21"/>
+      <c r="M14" s="21"/>
+      <c r="N14" s="21"/>
+      <c r="O14" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P14" s="28"/>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="28"/>
-      <c r="S14" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T14" s="28"/>
-      <c r="U14" s="28"/>
-      <c r="V14" s="28"/>
-      <c r="W14" s="28"/>
-      <c r="X14" s="28"/>
-      <c r="Y14" s="28"/>
-      <c r="Z14" s="28"/>
-      <c r="AA14" s="28"/>
-      <c r="AB14" s="28"/>
-      <c r="AC14" s="28"/>
-      <c r="AD14" s="28"/>
-      <c r="AE14" s="28"/>
-      <c r="AF14" s="28"/>
-      <c r="AG14" s="28"/>
-      <c r="AH14" s="29"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="21"/>
+      <c r="R14" s="21"/>
+      <c r="S14" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T14" s="21"/>
+      <c r="U14" s="21"/>
+      <c r="V14" s="21"/>
+      <c r="W14" s="21"/>
+      <c r="X14" s="21"/>
+      <c r="Y14" s="21"/>
+      <c r="Z14" s="21"/>
+      <c r="AA14" s="21"/>
+      <c r="AB14" s="21"/>
+      <c r="AC14" s="21"/>
+      <c r="AD14" s="21"/>
+      <c r="AE14" s="21"/>
+      <c r="AF14" s="21"/>
+      <c r="AG14" s="21"/>
+      <c r="AH14" s="30"/>
     </row>
-    <row r="15" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
@@ -2585,43 +2595,43 @@
       <c r="J15" s="6">
         <v>0</v>
       </c>
-      <c r="K15" s="23" t="s">
+      <c r="K15" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L15" s="28"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28"/>
-      <c r="O15" s="28" t="s">
+      <c r="L15" s="21"/>
+      <c r="M15" s="21"/>
+      <c r="N15" s="21"/>
+      <c r="O15" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P15" s="28"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="28"/>
-      <c r="S15" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T15" s="28"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
-      <c r="W15" s="28"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
-      <c r="Z15" s="28"/>
-      <c r="AA15" s="28"/>
-      <c r="AB15" s="28"/>
-      <c r="AC15" s="28"/>
-      <c r="AD15" s="28"/>
-      <c r="AE15" s="28"/>
-      <c r="AF15" s="28"/>
-      <c r="AG15" s="28"/>
-      <c r="AH15" s="29"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
+      <c r="S15" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T15" s="21"/>
+      <c r="U15" s="21"/>
+      <c r="V15" s="21"/>
+      <c r="W15" s="21"/>
+      <c r="X15" s="21"/>
+      <c r="Y15" s="21"/>
+      <c r="Z15" s="21"/>
+      <c r="AA15" s="21"/>
+      <c r="AB15" s="21"/>
+      <c r="AC15" s="21"/>
+      <c r="AD15" s="21"/>
+      <c r="AE15" s="21"/>
+      <c r="AF15" s="21"/>
+      <c r="AG15" s="21"/>
+      <c r="AH15" s="30"/>
     </row>
-    <row r="16" spans="1:38" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:38" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C16" s="5">
         <v>1</v>
@@ -2647,105 +2657,105 @@
       <c r="J16" s="6">
         <v>0</v>
       </c>
-      <c r="K16" s="23" t="s">
+      <c r="K16" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L16" s="28"/>
-      <c r="M16" s="28"/>
-      <c r="N16" s="28"/>
-      <c r="O16" s="28" t="s">
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P16" s="28"/>
-      <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
-      <c r="S16" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T16" s="28"/>
-      <c r="U16" s="28"/>
-      <c r="V16" s="28"/>
-      <c r="W16" s="28"/>
-      <c r="X16" s="28"/>
-      <c r="Y16" s="28"/>
-      <c r="Z16" s="28"/>
-      <c r="AA16" s="28"/>
-      <c r="AB16" s="28"/>
-      <c r="AC16" s="28"/>
-      <c r="AD16" s="28"/>
-      <c r="AE16" s="28"/>
-      <c r="AF16" s="28"/>
-      <c r="AG16" s="28"/>
-      <c r="AH16" s="29"/>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="21"/>
+      <c r="R16" s="21"/>
+      <c r="S16" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T16" s="21"/>
+      <c r="U16" s="21"/>
+      <c r="V16" s="21"/>
+      <c r="W16" s="21"/>
+      <c r="X16" s="21"/>
+      <c r="Y16" s="21"/>
+      <c r="Z16" s="21"/>
+      <c r="AA16" s="21"/>
+      <c r="AB16" s="21"/>
+      <c r="AC16" s="21"/>
+      <c r="AD16" s="21"/>
+      <c r="AE16" s="21"/>
+      <c r="AF16" s="21"/>
+      <c r="AG16" s="21"/>
+      <c r="AH16" s="30"/>
     </row>
-    <row r="17" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>1</v>
+      </c>
+      <c r="J17" s="6">
+        <v>0</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+      <c r="O17" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="P17" s="21"/>
+      <c r="Q17" s="21"/>
+      <c r="R17" s="21"/>
+      <c r="S17" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="5">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1">
-        <v>0</v>
-      </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
-      <c r="F17" s="1">
-        <v>1</v>
-      </c>
-      <c r="G17" s="1">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>0</v>
-      </c>
-      <c r="I17" s="5">
-        <v>1</v>
-      </c>
-      <c r="J17" s="6">
-        <v>0</v>
-      </c>
-      <c r="K17" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="L17" s="28"/>
-      <c r="M17" s="28"/>
-      <c r="N17" s="28"/>
-      <c r="O17" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="P17" s="28"/>
-      <c r="Q17" s="28"/>
-      <c r="R17" s="28"/>
-      <c r="S17" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T17" s="28"/>
-      <c r="U17" s="28"/>
-      <c r="V17" s="28"/>
-      <c r="W17" s="28"/>
-      <c r="X17" s="28"/>
-      <c r="Y17" s="28"/>
-      <c r="Z17" s="28"/>
-      <c r="AA17" s="28"/>
-      <c r="AB17" s="28"/>
-      <c r="AC17" s="28"/>
-      <c r="AD17" s="28"/>
-      <c r="AE17" s="28"/>
-      <c r="AF17" s="28"/>
-      <c r="AG17" s="28"/>
-      <c r="AH17" s="29"/>
+      <c r="T17" s="21"/>
+      <c r="U17" s="21"/>
+      <c r="V17" s="21"/>
+      <c r="W17" s="21"/>
+      <c r="X17" s="21"/>
+      <c r="Y17" s="21"/>
+      <c r="Z17" s="21"/>
+      <c r="AA17" s="21"/>
+      <c r="AB17" s="21"/>
+      <c r="AC17" s="21"/>
+      <c r="AD17" s="21"/>
+      <c r="AE17" s="21"/>
+      <c r="AF17" s="21"/>
+      <c r="AG17" s="21"/>
+      <c r="AH17" s="30"/>
     </row>
-    <row r="18" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
@@ -2771,43 +2781,43 @@
       <c r="J18" s="6">
         <v>0</v>
       </c>
-      <c r="K18" s="23" t="s">
+      <c r="K18" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L18" s="28"/>
-      <c r="M18" s="28"/>
-      <c r="N18" s="28"/>
-      <c r="O18" s="28" t="s">
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P18" s="28"/>
-      <c r="Q18" s="28"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
-      <c r="V18" s="28"/>
-      <c r="W18" s="28"/>
-      <c r="X18" s="28"/>
-      <c r="Y18" s="28"/>
-      <c r="Z18" s="28"/>
-      <c r="AA18" s="28"/>
-      <c r="AB18" s="28"/>
-      <c r="AC18" s="28"/>
-      <c r="AD18" s="28"/>
-      <c r="AE18" s="28"/>
-      <c r="AF18" s="28"/>
-      <c r="AG18" s="28"/>
-      <c r="AH18" s="29"/>
+      <c r="P18" s="21"/>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T18" s="21"/>
+      <c r="U18" s="21"/>
+      <c r="V18" s="21"/>
+      <c r="W18" s="21"/>
+      <c r="X18" s="21"/>
+      <c r="Y18" s="21"/>
+      <c r="Z18" s="21"/>
+      <c r="AA18" s="21"/>
+      <c r="AB18" s="21"/>
+      <c r="AC18" s="21"/>
+      <c r="AD18" s="21"/>
+      <c r="AE18" s="21"/>
+      <c r="AF18" s="21"/>
+      <c r="AG18" s="21"/>
+      <c r="AH18" s="30"/>
     </row>
-    <row r="19" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -2833,43 +2843,43 @@
       <c r="J19" s="6">
         <v>0</v>
       </c>
-      <c r="K19" s="23" t="s">
+      <c r="K19" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
-      <c r="O19" s="28" t="s">
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P19" s="28"/>
-      <c r="Q19" s="28"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
-      <c r="V19" s="28"/>
-      <c r="W19" s="28"/>
-      <c r="X19" s="28"/>
-      <c r="Y19" s="28"/>
-      <c r="Z19" s="28"/>
-      <c r="AA19" s="28"/>
-      <c r="AB19" s="28"/>
-      <c r="AC19" s="28"/>
-      <c r="AD19" s="28"/>
-      <c r="AE19" s="28"/>
-      <c r="AF19" s="28"/>
-      <c r="AG19" s="28"/>
-      <c r="AH19" s="29"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T19" s="21"/>
+      <c r="U19" s="21"/>
+      <c r="V19" s="21"/>
+      <c r="W19" s="21"/>
+      <c r="X19" s="21"/>
+      <c r="Y19" s="21"/>
+      <c r="Z19" s="21"/>
+      <c r="AA19" s="21"/>
+      <c r="AB19" s="21"/>
+      <c r="AC19" s="21"/>
+      <c r="AD19" s="21"/>
+      <c r="AE19" s="21"/>
+      <c r="AF19" s="21"/>
+      <c r="AG19" s="21"/>
+      <c r="AH19" s="30"/>
     </row>
-    <row r="20" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C20" s="5">
         <v>1</v>
@@ -2895,38 +2905,38 @@
       <c r="J20" s="6">
         <v>0</v>
       </c>
-      <c r="K20" s="23" t="s">
+      <c r="K20" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28" t="s">
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
-      <c r="V20" s="28"/>
-      <c r="W20" s="28"/>
-      <c r="X20" s="28"/>
-      <c r="Y20" s="28"/>
-      <c r="Z20" s="28"/>
-      <c r="AA20" s="28"/>
-      <c r="AB20" s="28"/>
-      <c r="AC20" s="28"/>
-      <c r="AD20" s="28"/>
-      <c r="AE20" s="28"/>
-      <c r="AF20" s="28"/>
-      <c r="AG20" s="28"/>
-      <c r="AH20" s="29"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T20" s="21"/>
+      <c r="U20" s="21"/>
+      <c r="V20" s="21"/>
+      <c r="W20" s="21"/>
+      <c r="X20" s="21"/>
+      <c r="Y20" s="21"/>
+      <c r="Z20" s="21"/>
+      <c r="AA20" s="21"/>
+      <c r="AB20" s="21"/>
+      <c r="AC20" s="21"/>
+      <c r="AD20" s="21"/>
+      <c r="AE20" s="21"/>
+      <c r="AF20" s="21"/>
+      <c r="AG20" s="21"/>
+      <c r="AH20" s="30"/>
     </row>
-    <row r="21" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="5" t="s">
         <v>56</v>
       </c>
@@ -2957,40 +2967,40 @@
       <c r="J21" s="6">
         <v>0</v>
       </c>
-      <c r="K21" s="23" t="s">
+      <c r="K21" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28" t="s">
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P21" s="28"/>
-      <c r="Q21" s="28"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="33">
-        <v>0</v>
-      </c>
-      <c r="T21" s="33"/>
-      <c r="U21" s="33"/>
-      <c r="V21" s="33"/>
-      <c r="W21" s="33"/>
-      <c r="X21" s="33"/>
-      <c r="Y21" s="33"/>
-      <c r="Z21" s="33"/>
-      <c r="AA21" s="33"/>
-      <c r="AB21" s="33"/>
-      <c r="AC21" s="33"/>
-      <c r="AD21" s="33"/>
-      <c r="AE21" s="28" t="s">
+      <c r="P21" s="21"/>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="21"/>
+      <c r="S21" s="22">
+        <v>0</v>
+      </c>
+      <c r="T21" s="22"/>
+      <c r="U21" s="22"/>
+      <c r="V21" s="22"/>
+      <c r="W21" s="22"/>
+      <c r="X21" s="22"/>
+      <c r="Y21" s="22"/>
+      <c r="Z21" s="22"/>
+      <c r="AA21" s="22"/>
+      <c r="AB21" s="22"/>
+      <c r="AC21" s="22"/>
+      <c r="AD21" s="22"/>
+      <c r="AE21" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="AF21" s="28"/>
-      <c r="AG21" s="28"/>
-      <c r="AH21" s="29"/>
+      <c r="AF21" s="21"/>
+      <c r="AG21" s="21"/>
+      <c r="AH21" s="30"/>
     </row>
-    <row r="22" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="5" t="s">
         <v>57</v>
       </c>
@@ -3021,40 +3031,40 @@
       <c r="J22" s="6">
         <v>0</v>
       </c>
-      <c r="K22" s="23" t="s">
+      <c r="K22" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28" t="s">
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P22" s="28"/>
-      <c r="Q22" s="28"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="33">
-        <v>0</v>
-      </c>
-      <c r="T22" s="33"/>
-      <c r="U22" s="33"/>
-      <c r="V22" s="33"/>
-      <c r="W22" s="33"/>
-      <c r="X22" s="33"/>
-      <c r="Y22" s="33"/>
-      <c r="Z22" s="33"/>
-      <c r="AA22" s="33"/>
-      <c r="AB22" s="33"/>
-      <c r="AC22" s="33"/>
-      <c r="AD22" s="33"/>
-      <c r="AE22" s="28" t="s">
+      <c r="P22" s="21"/>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="22">
+        <v>0</v>
+      </c>
+      <c r="T22" s="22"/>
+      <c r="U22" s="22"/>
+      <c r="V22" s="22"/>
+      <c r="W22" s="22"/>
+      <c r="X22" s="22"/>
+      <c r="Y22" s="22"/>
+      <c r="Z22" s="22"/>
+      <c r="AA22" s="22"/>
+      <c r="AB22" s="22"/>
+      <c r="AC22" s="22"/>
+      <c r="AD22" s="22"/>
+      <c r="AE22" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="AF22" s="28"/>
-      <c r="AG22" s="28"/>
-      <c r="AH22" s="29"/>
+      <c r="AF22" s="21"/>
+      <c r="AG22" s="21"/>
+      <c r="AH22" s="30"/>
     </row>
-    <row r="23" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="5" t="s">
         <v>58</v>
       </c>
@@ -3085,40 +3095,40 @@
       <c r="J23" s="6">
         <v>0</v>
       </c>
-      <c r="K23" s="23" t="s">
+      <c r="K23" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L23" s="28"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
-      <c r="O23" s="28" t="s">
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P23" s="28"/>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="33">
-        <v>0</v>
-      </c>
-      <c r="T23" s="33"/>
-      <c r="U23" s="33"/>
-      <c r="V23" s="33"/>
-      <c r="W23" s="33"/>
-      <c r="X23" s="33"/>
-      <c r="Y23" s="33"/>
-      <c r="Z23" s="33"/>
-      <c r="AA23" s="33"/>
-      <c r="AB23" s="33"/>
-      <c r="AC23" s="33"/>
-      <c r="AD23" s="33"/>
-      <c r="AE23" s="28" t="s">
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="22">
+        <v>0</v>
+      </c>
+      <c r="T23" s="22"/>
+      <c r="U23" s="22"/>
+      <c r="V23" s="22"/>
+      <c r="W23" s="22"/>
+      <c r="X23" s="22"/>
+      <c r="Y23" s="22"/>
+      <c r="Z23" s="22"/>
+      <c r="AA23" s="22"/>
+      <c r="AB23" s="22"/>
+      <c r="AC23" s="22"/>
+      <c r="AD23" s="22"/>
+      <c r="AE23" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="AF23" s="28"/>
-      <c r="AG23" s="28"/>
-      <c r="AH23" s="29"/>
+      <c r="AF23" s="21"/>
+      <c r="AG23" s="21"/>
+      <c r="AH23" s="30"/>
     </row>
-    <row r="24" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>59</v>
       </c>
@@ -3149,40 +3159,40 @@
       <c r="J24" s="6">
         <v>0</v>
       </c>
-      <c r="K24" s="23" t="s">
+      <c r="K24" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L24" s="28"/>
-      <c r="M24" s="28"/>
-      <c r="N24" s="28"/>
-      <c r="O24" s="28" t="s">
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P24" s="28"/>
-      <c r="Q24" s="28"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28" t="s">
+      <c r="P24" s="21"/>
+      <c r="Q24" s="21"/>
+      <c r="R24" s="21"/>
+      <c r="S24" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
-      <c r="V24" s="28"/>
-      <c r="W24" s="33">
-        <v>0</v>
-      </c>
-      <c r="X24" s="33"/>
-      <c r="Y24" s="33"/>
-      <c r="Z24" s="33"/>
-      <c r="AA24" s="33"/>
-      <c r="AB24" s="33"/>
-      <c r="AC24" s="33"/>
-      <c r="AD24" s="33"/>
-      <c r="AE24" s="33"/>
-      <c r="AF24" s="33"/>
-      <c r="AG24" s="33"/>
-      <c r="AH24" s="34"/>
+      <c r="T24" s="21"/>
+      <c r="U24" s="21"/>
+      <c r="V24" s="21"/>
+      <c r="W24" s="22">
+        <v>0</v>
+      </c>
+      <c r="X24" s="22"/>
+      <c r="Y24" s="22"/>
+      <c r="Z24" s="22"/>
+      <c r="AA24" s="22"/>
+      <c r="AB24" s="22"/>
+      <c r="AC24" s="22"/>
+      <c r="AD24" s="22"/>
+      <c r="AE24" s="22"/>
+      <c r="AF24" s="22"/>
+      <c r="AG24" s="22"/>
+      <c r="AH24" s="23"/>
     </row>
-    <row r="25" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="5" t="s">
         <v>60</v>
       </c>
@@ -3213,40 +3223,40 @@
       <c r="J25" s="6">
         <v>0</v>
       </c>
-      <c r="K25" s="23" t="s">
+      <c r="K25" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-      <c r="O25" s="28" t="s">
+      <c r="L25" s="21"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P25" s="28"/>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28" t="s">
+      <c r="P25" s="21"/>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="21"/>
+      <c r="S25" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="28"/>
-      <c r="W25" s="33">
-        <v>0</v>
-      </c>
-      <c r="X25" s="33"/>
-      <c r="Y25" s="33"/>
-      <c r="Z25" s="33"/>
-      <c r="AA25" s="33"/>
-      <c r="AB25" s="33"/>
-      <c r="AC25" s="33"/>
-      <c r="AD25" s="33"/>
-      <c r="AE25" s="33"/>
-      <c r="AF25" s="33"/>
-      <c r="AG25" s="33"/>
-      <c r="AH25" s="34"/>
+      <c r="T25" s="21"/>
+      <c r="U25" s="21"/>
+      <c r="V25" s="21"/>
+      <c r="W25" s="22">
+        <v>0</v>
+      </c>
+      <c r="X25" s="22"/>
+      <c r="Y25" s="22"/>
+      <c r="Z25" s="22"/>
+      <c r="AA25" s="22"/>
+      <c r="AB25" s="22"/>
+      <c r="AC25" s="22"/>
+      <c r="AD25" s="22"/>
+      <c r="AE25" s="22"/>
+      <c r="AF25" s="22"/>
+      <c r="AG25" s="22"/>
+      <c r="AH25" s="23"/>
     </row>
-    <row r="26" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="5" t="s">
         <v>61</v>
       </c>
@@ -3277,298 +3287,298 @@
       <c r="J26" s="6">
         <v>0</v>
       </c>
-      <c r="K26" s="23" t="s">
+      <c r="K26" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L26" s="28"/>
-      <c r="M26" s="28"/>
-      <c r="N26" s="28"/>
-      <c r="O26" s="28" t="s">
+      <c r="L26" s="21"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="21"/>
+      <c r="O26" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P26" s="28"/>
-      <c r="Q26" s="28"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28" t="s">
+      <c r="P26" s="21"/>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="21"/>
+      <c r="S26" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
-      <c r="V26" s="28"/>
-      <c r="W26" s="33">
-        <v>0</v>
-      </c>
-      <c r="X26" s="33"/>
-      <c r="Y26" s="33"/>
-      <c r="Z26" s="33"/>
-      <c r="AA26" s="33"/>
-      <c r="AB26" s="33"/>
-      <c r="AC26" s="33"/>
-      <c r="AD26" s="33"/>
-      <c r="AE26" s="33"/>
-      <c r="AF26" s="33"/>
-      <c r="AG26" s="33"/>
-      <c r="AH26" s="34"/>
+      <c r="T26" s="21"/>
+      <c r="U26" s="21"/>
+      <c r="V26" s="21"/>
+      <c r="W26" s="22">
+        <v>0</v>
+      </c>
+      <c r="X26" s="22"/>
+      <c r="Y26" s="22"/>
+      <c r="Z26" s="22"/>
+      <c r="AA26" s="22"/>
+      <c r="AB26" s="22"/>
+      <c r="AC26" s="22"/>
+      <c r="AD26" s="22"/>
+      <c r="AE26" s="22"/>
+      <c r="AF26" s="22"/>
+      <c r="AG26" s="22"/>
+      <c r="AH26" s="23"/>
     </row>
-    <row r="27" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+      <c r="H27" s="6">
+        <v>0</v>
+      </c>
+      <c r="I27" s="5">
+        <v>0</v>
+      </c>
+      <c r="J27" s="6">
+        <v>1</v>
+      </c>
+      <c r="K27" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="P27" s="21"/>
+      <c r="Q27" s="21"/>
+      <c r="R27" s="21"/>
+      <c r="S27" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="T27" s="21"/>
+      <c r="U27" s="21"/>
+      <c r="V27" s="21"/>
+      <c r="W27" s="22">
+        <v>0</v>
+      </c>
+      <c r="X27" s="22"/>
+      <c r="Y27" s="22"/>
+      <c r="Z27" s="22"/>
+      <c r="AA27" s="22"/>
+      <c r="AB27" s="22"/>
+      <c r="AC27" s="22"/>
+      <c r="AD27" s="22"/>
+      <c r="AE27" s="22"/>
+      <c r="AF27" s="22"/>
+      <c r="AG27" s="22"/>
+      <c r="AH27" s="23"/>
+    </row>
+    <row r="28" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="5">
+        <v>1</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0</v>
+      </c>
+      <c r="F28" s="1">
+        <v>0</v>
+      </c>
+      <c r="G28" s="1">
+        <v>0</v>
+      </c>
+      <c r="H28" s="6">
+        <v>1</v>
+      </c>
+      <c r="I28" s="5">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6">
+        <v>1</v>
+      </c>
+      <c r="K28" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="P28" s="21"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="21"/>
+      <c r="S28" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="T28" s="21"/>
+      <c r="U28" s="21"/>
+      <c r="V28" s="21"/>
+      <c r="W28" s="22">
+        <v>0</v>
+      </c>
+      <c r="X28" s="22"/>
+      <c r="Y28" s="22"/>
+      <c r="Z28" s="22"/>
+      <c r="AA28" s="22"/>
+      <c r="AB28" s="22"/>
+      <c r="AC28" s="22"/>
+      <c r="AD28" s="22"/>
+      <c r="AE28" s="22"/>
+      <c r="AF28" s="22"/>
+      <c r="AG28" s="22"/>
+      <c r="AH28" s="23"/>
+    </row>
+    <row r="29" spans="1:37" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B29" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="5">
-        <v>1</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0</v>
-      </c>
-      <c r="E27" s="1">
-        <v>0</v>
-      </c>
-      <c r="F27" s="1">
-        <v>0</v>
-      </c>
-      <c r="G27" s="1">
-        <v>0</v>
-      </c>
-      <c r="H27" s="6">
-        <v>0</v>
-      </c>
-      <c r="I27" s="5">
-        <v>0</v>
-      </c>
-      <c r="J27" s="6">
-        <v>1</v>
-      </c>
-      <c r="K27" s="23" t="s">
+      <c r="C29" s="5">
+        <v>1</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0</v>
+      </c>
+      <c r="E29" s="1">
+        <v>0</v>
+      </c>
+      <c r="F29" s="1">
+        <v>0</v>
+      </c>
+      <c r="G29" s="1">
+        <v>0</v>
+      </c>
+      <c r="H29" s="6">
+        <v>0</v>
+      </c>
+      <c r="I29" s="5">
+        <v>1</v>
+      </c>
+      <c r="J29" s="6">
+        <v>1</v>
+      </c>
+      <c r="K29" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L27" s="28"/>
-      <c r="M27" s="28"/>
-      <c r="N27" s="28"/>
-      <c r="O27" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="P27" s="28"/>
-      <c r="Q27" s="28"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
-      <c r="V27" s="28"/>
-      <c r="W27" s="33">
-        <v>0</v>
-      </c>
-      <c r="X27" s="33"/>
-      <c r="Y27" s="33"/>
-      <c r="Z27" s="33"/>
-      <c r="AA27" s="33"/>
-      <c r="AB27" s="33"/>
-      <c r="AC27" s="33"/>
-      <c r="AD27" s="33"/>
-      <c r="AE27" s="33"/>
-      <c r="AF27" s="33"/>
-      <c r="AG27" s="33"/>
-      <c r="AH27" s="34"/>
+      <c r="L29" s="21"/>
+      <c r="M29" s="21"/>
+      <c r="N29" s="21"/>
+      <c r="O29" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="P29" s="21"/>
+      <c r="Q29" s="21"/>
+      <c r="R29" s="21"/>
+      <c r="S29" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T29" s="21"/>
+      <c r="U29" s="21"/>
+      <c r="V29" s="21"/>
+      <c r="W29" s="21"/>
+      <c r="X29" s="21"/>
+      <c r="Y29" s="21"/>
+      <c r="Z29" s="21"/>
+      <c r="AA29" s="21"/>
+      <c r="AB29" s="21"/>
+      <c r="AC29" s="21"/>
+      <c r="AD29" s="21"/>
+      <c r="AE29" s="21"/>
+      <c r="AF29" s="21"/>
+      <c r="AG29" s="21"/>
+      <c r="AH29" s="30"/>
     </row>
-    <row r="28" spans="1:37" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="5" t="s">
+    <row r="30" spans="1:37" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B30" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="5">
-        <v>1</v>
-      </c>
-      <c r="D28" s="1">
-        <v>0</v>
-      </c>
-      <c r="E28" s="1">
-        <v>0</v>
-      </c>
-      <c r="F28" s="1">
-        <v>0</v>
-      </c>
-      <c r="G28" s="1">
-        <v>0</v>
-      </c>
-      <c r="H28" s="6">
-        <v>1</v>
-      </c>
-      <c r="I28" s="5">
-        <v>0</v>
-      </c>
-      <c r="J28" s="6">
-        <v>1</v>
-      </c>
-      <c r="K28" s="23" t="s">
+      <c r="C30" s="5">
+        <v>1</v>
+      </c>
+      <c r="D30" s="1">
+        <v>0</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1">
+        <v>0</v>
+      </c>
+      <c r="H30" s="6">
+        <v>1</v>
+      </c>
+      <c r="I30" s="5">
+        <v>1</v>
+      </c>
+      <c r="J30" s="6">
+        <v>1</v>
+      </c>
+      <c r="K30" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L28" s="28"/>
-      <c r="M28" s="28"/>
-      <c r="N28" s="28"/>
-      <c r="O28" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
-      <c r="V28" s="28"/>
-      <c r="W28" s="33">
-        <v>0</v>
-      </c>
-      <c r="X28" s="33"/>
-      <c r="Y28" s="33"/>
-      <c r="Z28" s="33"/>
-      <c r="AA28" s="33"/>
-      <c r="AB28" s="33"/>
-      <c r="AC28" s="33"/>
-      <c r="AD28" s="33"/>
-      <c r="AE28" s="33"/>
-      <c r="AF28" s="33"/>
-      <c r="AG28" s="33"/>
-      <c r="AH28" s="34"/>
-    </row>
-    <row r="29" spans="1:37" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C29" s="5">
-        <v>1</v>
-      </c>
-      <c r="D29" s="1">
-        <v>0</v>
-      </c>
-      <c r="E29" s="1">
-        <v>0</v>
-      </c>
-      <c r="F29" s="1">
-        <v>0</v>
-      </c>
-      <c r="G29" s="1">
-        <v>0</v>
-      </c>
-      <c r="H29" s="6">
-        <v>0</v>
-      </c>
-      <c r="I29" s="5">
-        <v>1</v>
-      </c>
-      <c r="J29" s="6">
-        <v>1</v>
-      </c>
-      <c r="K29" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28" t="s">
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
-      <c r="V29" s="28"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="28"/>
-      <c r="AB29" s="28"/>
-      <c r="AC29" s="28"/>
-      <c r="AD29" s="28"/>
-      <c r="AE29" s="28"/>
-      <c r="AF29" s="28"/>
-      <c r="AG29" s="28"/>
-      <c r="AH29" s="29"/>
-    </row>
-    <row r="30" spans="1:37" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C30" s="5">
-        <v>1</v>
-      </c>
-      <c r="D30" s="1">
-        <v>0</v>
-      </c>
-      <c r="E30" s="1">
-        <v>0</v>
-      </c>
-      <c r="F30" s="1">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1">
-        <v>0</v>
-      </c>
-      <c r="H30" s="6">
-        <v>1</v>
-      </c>
-      <c r="I30" s="5">
-        <v>1</v>
-      </c>
-      <c r="J30" s="6">
-        <v>1</v>
-      </c>
-      <c r="K30" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="L30" s="28"/>
-      <c r="M30" s="28"/>
-      <c r="N30" s="28"/>
-      <c r="O30" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
-      <c r="V30" s="28"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
-      <c r="Z30" s="28"/>
-      <c r="AA30" s="28"/>
-      <c r="AB30" s="28"/>
-      <c r="AC30" s="28"/>
-      <c r="AD30" s="28"/>
-      <c r="AE30" s="28"/>
-      <c r="AF30" s="28"/>
-      <c r="AG30" s="28"/>
-      <c r="AH30" s="29"/>
+      <c r="P30" s="21"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T30" s="21"/>
+      <c r="U30" s="21"/>
+      <c r="V30" s="21"/>
+      <c r="W30" s="21"/>
+      <c r="X30" s="21"/>
+      <c r="Y30" s="21"/>
+      <c r="Z30" s="21"/>
+      <c r="AA30" s="21"/>
+      <c r="AB30" s="21"/>
+      <c r="AC30" s="21"/>
+      <c r="AD30" s="21"/>
+      <c r="AE30" s="21"/>
+      <c r="AF30" s="21"/>
+      <c r="AG30" s="21"/>
+      <c r="AH30" s="30"/>
       <c r="AJ30" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="AK30" s="13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="39" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>51</v>
       </c>
@@ -3602,43 +3612,43 @@
       <c r="K31" s="27">
         <v>0</v>
       </c>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-      <c r="O31" s="28" t="s">
+      <c r="L31" s="22"/>
+      <c r="M31" s="22"/>
+      <c r="N31" s="22"/>
+      <c r="O31" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P31" s="28"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28" t="s">
+      <c r="P31" s="21"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
-      <c r="V31" s="28"/>
-      <c r="W31" s="33">
-        <v>0</v>
-      </c>
-      <c r="X31" s="33"/>
-      <c r="Y31" s="33"/>
-      <c r="Z31" s="33"/>
-      <c r="AA31" s="33"/>
-      <c r="AB31" s="33"/>
-      <c r="AC31" s="33"/>
-      <c r="AD31" s="33"/>
-      <c r="AE31" s="33"/>
-      <c r="AF31" s="33"/>
-      <c r="AG31" s="33"/>
-      <c r="AH31" s="34"/>
+      <c r="T31" s="21"/>
+      <c r="U31" s="21"/>
+      <c r="V31" s="21"/>
+      <c r="W31" s="22">
+        <v>0</v>
+      </c>
+      <c r="X31" s="22"/>
+      <c r="Y31" s="22"/>
+      <c r="Z31" s="22"/>
+      <c r="AA31" s="22"/>
+      <c r="AB31" s="22"/>
+      <c r="AC31" s="22"/>
+      <c r="AD31" s="22"/>
+      <c r="AE31" s="22"/>
+      <c r="AF31" s="22"/>
+      <c r="AG31" s="22"/>
+      <c r="AH31" s="23"/>
       <c r="AJ31" s="10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="AK31" s="11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="39" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="5" t="s">
         <v>52</v>
       </c>
@@ -3672,48 +3682,48 @@
       <c r="K32" s="27">
         <v>0</v>
       </c>
-      <c r="L32" s="33"/>
-      <c r="M32" s="33"/>
-      <c r="N32" s="33"/>
-      <c r="O32" s="28" t="s">
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28" t="s">
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
-      <c r="W32" s="33">
-        <v>0</v>
-      </c>
-      <c r="X32" s="33"/>
-      <c r="Y32" s="33"/>
-      <c r="Z32" s="33"/>
-      <c r="AA32" s="33"/>
-      <c r="AB32" s="33"/>
-      <c r="AC32" s="33"/>
-      <c r="AD32" s="33"/>
-      <c r="AE32" s="33"/>
-      <c r="AF32" s="33"/>
-      <c r="AG32" s="33"/>
-      <c r="AH32" s="34"/>
+      <c r="T32" s="21"/>
+      <c r="U32" s="21"/>
+      <c r="V32" s="21"/>
+      <c r="W32" s="22">
+        <v>0</v>
+      </c>
+      <c r="X32" s="22"/>
+      <c r="Y32" s="22"/>
+      <c r="Z32" s="22"/>
+      <c r="AA32" s="22"/>
+      <c r="AB32" s="22"/>
+      <c r="AC32" s="22"/>
+      <c r="AD32" s="22"/>
+      <c r="AE32" s="22"/>
+      <c r="AF32" s="22"/>
+      <c r="AG32" s="22"/>
+      <c r="AH32" s="23"/>
       <c r="AJ32" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="AK32" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:43" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C33" s="5">
         <v>0</v>
@@ -3745,12 +3755,12 @@
       <c r="L33" s="25"/>
       <c r="M33" s="25"/>
       <c r="N33" s="27"/>
-      <c r="O33" s="38" t="s">
+      <c r="O33" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="P33" s="22"/>
-      <c r="Q33" s="22"/>
-      <c r="R33" s="23"/>
+      <c r="P33" s="29"/>
+      <c r="Q33" s="29"/>
+      <c r="R33" s="20"/>
       <c r="S33" s="24">
         <v>0</v>
       </c>
@@ -3769,19 +3779,19 @@
       <c r="AF33" s="25"/>
       <c r="AG33" s="25"/>
       <c r="AH33" s="26"/>
-      <c r="AJ33" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="AK33" s="8" t="s">
-        <v>113</v>
+      <c r="AJ33" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK33" s="49" t="s">
+        <v>142</v>
       </c>
     </row>
-    <row r="34" spans="1:43" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:43" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C34" s="5">
         <v>1</v>
@@ -3807,43 +3817,49 @@
       <c r="J34" s="6">
         <v>0</v>
       </c>
-      <c r="K34" s="23" t="s">
+      <c r="K34" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L34" s="28"/>
-      <c r="M34" s="28"/>
-      <c r="N34" s="28"/>
+      <c r="L34" s="21"/>
+      <c r="M34" s="21"/>
+      <c r="N34" s="21"/>
       <c r="O34" s="25">
         <v>0</v>
       </c>
       <c r="P34" s="25"/>
       <c r="Q34" s="25"/>
       <c r="R34" s="27"/>
-      <c r="S34" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
-      <c r="V34" s="28"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
-      <c r="AC34" s="28"/>
-      <c r="AD34" s="28"/>
-      <c r="AE34" s="28"/>
-      <c r="AF34" s="28"/>
-      <c r="AG34" s="28"/>
-      <c r="AH34" s="29"/>
+      <c r="S34" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T34" s="21"/>
+      <c r="U34" s="21"/>
+      <c r="V34" s="21"/>
+      <c r="W34" s="21"/>
+      <c r="X34" s="21"/>
+      <c r="Y34" s="21"/>
+      <c r="Z34" s="21"/>
+      <c r="AA34" s="21"/>
+      <c r="AB34" s="21"/>
+      <c r="AC34" s="21"/>
+      <c r="AD34" s="21"/>
+      <c r="AE34" s="21"/>
+      <c r="AF34" s="21"/>
+      <c r="AG34" s="21"/>
+      <c r="AH34" s="30"/>
+      <c r="AJ34" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="AK34" s="8" t="s">
+        <v>109</v>
+      </c>
     </row>
-    <row r="35" spans="1:43" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C35" s="5">
         <v>1</v>
@@ -3869,43 +3885,43 @@
       <c r="J35" s="6">
         <v>0</v>
       </c>
-      <c r="K35" s="23" t="s">
+      <c r="K35" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L35" s="28"/>
-      <c r="M35" s="28"/>
-      <c r="N35" s="28"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="21"/>
+      <c r="N35" s="21"/>
       <c r="O35" s="25">
         <v>0</v>
       </c>
       <c r="P35" s="25"/>
       <c r="Q35" s="25"/>
       <c r="R35" s="27"/>
-      <c r="S35" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
-      <c r="V35" s="28"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
-      <c r="Z35" s="28"/>
-      <c r="AA35" s="28"/>
-      <c r="AB35" s="28"/>
-      <c r="AC35" s="28"/>
-      <c r="AD35" s="28"/>
-      <c r="AE35" s="28"/>
-      <c r="AF35" s="28"/>
-      <c r="AG35" s="28"/>
-      <c r="AH35" s="29"/>
+      <c r="S35" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T35" s="21"/>
+      <c r="U35" s="21"/>
+      <c r="V35" s="21"/>
+      <c r="W35" s="21"/>
+      <c r="X35" s="21"/>
+      <c r="Y35" s="21"/>
+      <c r="Z35" s="21"/>
+      <c r="AA35" s="21"/>
+      <c r="AB35" s="21"/>
+      <c r="AC35" s="21"/>
+      <c r="AD35" s="21"/>
+      <c r="AE35" s="21"/>
+      <c r="AF35" s="21"/>
+      <c r="AG35" s="21"/>
+      <c r="AH35" s="30"/>
     </row>
-    <row r="36" spans="1:43" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C36" s="5">
         <v>1</v>
@@ -3931,43 +3947,43 @@
       <c r="J36" s="6">
         <v>0</v>
       </c>
-      <c r="K36" s="21" t="s">
+      <c r="K36" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="L36" s="22"/>
-      <c r="M36" s="22"/>
-      <c r="N36" s="23"/>
+      <c r="L36" s="29"/>
+      <c r="M36" s="29"/>
+      <c r="N36" s="20"/>
       <c r="O36" s="25">
         <v>0</v>
       </c>
       <c r="P36" s="25"/>
       <c r="Q36" s="25"/>
       <c r="R36" s="27"/>
-      <c r="S36" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
-      <c r="V36" s="28"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
-      <c r="Z36" s="28"/>
-      <c r="AA36" s="28"/>
-      <c r="AB36" s="28"/>
-      <c r="AC36" s="28"/>
-      <c r="AD36" s="28"/>
-      <c r="AE36" s="28"/>
-      <c r="AF36" s="28"/>
-      <c r="AG36" s="28"/>
-      <c r="AH36" s="29"/>
+      <c r="S36" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T36" s="21"/>
+      <c r="U36" s="21"/>
+      <c r="V36" s="21"/>
+      <c r="W36" s="21"/>
+      <c r="X36" s="21"/>
+      <c r="Y36" s="21"/>
+      <c r="Z36" s="21"/>
+      <c r="AA36" s="21"/>
+      <c r="AB36" s="21"/>
+      <c r="AC36" s="21"/>
+      <c r="AD36" s="21"/>
+      <c r="AE36" s="21"/>
+      <c r="AF36" s="21"/>
+      <c r="AG36" s="21"/>
+      <c r="AH36" s="30"/>
     </row>
-    <row r="37" spans="1:43" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C37" s="5">
         <v>1</v>
@@ -3993,43 +4009,43 @@
       <c r="J37" s="6">
         <v>0</v>
       </c>
-      <c r="K37" s="21" t="s">
+      <c r="K37" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="L37" s="22"/>
-      <c r="M37" s="22"/>
-      <c r="N37" s="23"/>
+      <c r="L37" s="29"/>
+      <c r="M37" s="29"/>
+      <c r="N37" s="20"/>
       <c r="O37" s="25">
         <v>0</v>
       </c>
       <c r="P37" s="25"/>
       <c r="Q37" s="25"/>
       <c r="R37" s="27"/>
-      <c r="S37" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
-      <c r="V37" s="28"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
-      <c r="AC37" s="28"/>
-      <c r="AD37" s="28"/>
-      <c r="AE37" s="28"/>
-      <c r="AF37" s="28"/>
-      <c r="AG37" s="28"/>
-      <c r="AH37" s="29"/>
+      <c r="S37" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T37" s="21"/>
+      <c r="U37" s="21"/>
+      <c r="V37" s="21"/>
+      <c r="W37" s="21"/>
+      <c r="X37" s="21"/>
+      <c r="Y37" s="21"/>
+      <c r="Z37" s="21"/>
+      <c r="AA37" s="21"/>
+      <c r="AB37" s="21"/>
+      <c r="AC37" s="21"/>
+      <c r="AD37" s="21"/>
+      <c r="AE37" s="21"/>
+      <c r="AF37" s="21"/>
+      <c r="AG37" s="21"/>
+      <c r="AH37" s="30"/>
     </row>
-    <row r="38" spans="1:43" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C38" s="5">
         <v>1</v>
@@ -4055,45 +4071,43 @@
       <c r="J38" s="6">
         <v>0</v>
       </c>
-      <c r="K38" s="23" t="s">
+      <c r="K38" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
+      <c r="L38" s="21"/>
+      <c r="M38" s="21"/>
+      <c r="N38" s="21"/>
       <c r="O38" s="25">
         <v>0</v>
       </c>
       <c r="P38" s="25"/>
       <c r="Q38" s="25"/>
       <c r="R38" s="27"/>
-      <c r="S38" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
-      <c r="V38" s="28"/>
-      <c r="W38" s="28"/>
-      <c r="X38" s="28"/>
-      <c r="Y38" s="28"/>
-      <c r="Z38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="AC38" s="28"/>
-      <c r="AD38" s="28"/>
-      <c r="AE38" s="28"/>
-      <c r="AF38" s="28"/>
-      <c r="AG38" s="28"/>
-      <c r="AH38" s="29"/>
-      <c r="AJ38" s="3"/>
-      <c r="AK38" s="3"/>
+      <c r="S38" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T38" s="21"/>
+      <c r="U38" s="21"/>
+      <c r="V38" s="21"/>
+      <c r="W38" s="21"/>
+      <c r="X38" s="21"/>
+      <c r="Y38" s="21"/>
+      <c r="Z38" s="21"/>
+      <c r="AA38" s="21"/>
+      <c r="AB38" s="21"/>
+      <c r="AC38" s="21"/>
+      <c r="AD38" s="21"/>
+      <c r="AE38" s="21"/>
+      <c r="AF38" s="21"/>
+      <c r="AG38" s="21"/>
+      <c r="AH38" s="30"/>
     </row>
-    <row r="39" spans="1:43" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="5" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C39" s="5">
         <v>1</v>
@@ -4119,37 +4133,39 @@
       <c r="J39" s="6">
         <v>0</v>
       </c>
-      <c r="K39" s="23" t="s">
+      <c r="K39" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L39" s="28"/>
-      <c r="M39" s="28"/>
-      <c r="N39" s="28"/>
+      <c r="L39" s="21"/>
+      <c r="M39" s="21"/>
+      <c r="N39" s="21"/>
       <c r="O39" s="25">
         <v>0</v>
       </c>
       <c r="P39" s="25"/>
       <c r="Q39" s="25"/>
       <c r="R39" s="27"/>
-      <c r="S39" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="T39" s="28"/>
-      <c r="U39" s="28"/>
-      <c r="V39" s="28"/>
-      <c r="W39" s="28"/>
-      <c r="X39" s="28"/>
-      <c r="Y39" s="28"/>
-      <c r="Z39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-      <c r="AC39" s="28"/>
-      <c r="AD39" s="28"/>
-      <c r="AE39" s="28"/>
-      <c r="AF39" s="28"/>
-      <c r="AG39" s="28"/>
-      <c r="AH39" s="29"/>
+      <c r="S39" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="T39" s="21"/>
+      <c r="U39" s="21"/>
+      <c r="V39" s="21"/>
+      <c r="W39" s="21"/>
+      <c r="X39" s="21"/>
+      <c r="Y39" s="21"/>
+      <c r="Z39" s="21"/>
+      <c r="AA39" s="21"/>
+      <c r="AB39" s="21"/>
+      <c r="AC39" s="21"/>
+      <c r="AD39" s="21"/>
+      <c r="AE39" s="21"/>
+      <c r="AF39" s="21"/>
+      <c r="AG39" s="21"/>
+      <c r="AH39" s="30"/>
       <c r="AI39" s="3"/>
+      <c r="AJ39" s="3"/>
+      <c r="AK39" s="3"/>
       <c r="AL39" s="3"/>
       <c r="AM39" s="3"/>
       <c r="AN39" s="3"/>
@@ -4157,12 +4173,12 @@
       <c r="AP39" s="3"/>
       <c r="AQ39" s="3"/>
     </row>
-    <row r="40" spans="1:43" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="5" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C40" s="5">
         <v>1</v>
@@ -4188,12 +4204,12 @@
       <c r="J40" s="6">
         <v>0</v>
       </c>
-      <c r="K40" s="21" t="s">
+      <c r="K40" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="23"/>
+      <c r="L40" s="29"/>
+      <c r="M40" s="29"/>
+      <c r="N40" s="20"/>
       <c r="O40" s="24">
         <v>0</v>
       </c>
@@ -4224,12 +4240,12 @@
       <c r="AP40" s="3"/>
       <c r="AQ40" s="3"/>
     </row>
-    <row r="41" spans="1:43" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C41" s="5">
         <v>1</v>
@@ -4255,43 +4271,43 @@
       <c r="J41" s="6">
         <v>0</v>
       </c>
-      <c r="K41" s="23" t="s">
+      <c r="K41" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L41" s="28"/>
-      <c r="M41" s="28"/>
-      <c r="N41" s="28"/>
-      <c r="O41" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="P41" s="22"/>
-      <c r="Q41" s="22"/>
-      <c r="R41" s="23"/>
-      <c r="S41" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="T41" s="28"/>
-      <c r="U41" s="28"/>
-      <c r="V41" s="28"/>
-      <c r="W41" s="28"/>
-      <c r="X41" s="28"/>
-      <c r="Y41" s="28"/>
-      <c r="Z41" s="28"/>
-      <c r="AA41" s="28"/>
-      <c r="AB41" s="28"/>
-      <c r="AC41" s="28"/>
-      <c r="AD41" s="28"/>
-      <c r="AE41" s="28"/>
-      <c r="AF41" s="28"/>
-      <c r="AG41" s="28"/>
-      <c r="AH41" s="29"/>
+      <c r="L41" s="21"/>
+      <c r="M41" s="21"/>
+      <c r="N41" s="21"/>
+      <c r="O41" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="P41" s="29"/>
+      <c r="Q41" s="29"/>
+      <c r="R41" s="20"/>
+      <c r="S41" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="T41" s="21"/>
+      <c r="U41" s="21"/>
+      <c r="V41" s="21"/>
+      <c r="W41" s="21"/>
+      <c r="X41" s="21"/>
+      <c r="Y41" s="21"/>
+      <c r="Z41" s="21"/>
+      <c r="AA41" s="21"/>
+      <c r="AB41" s="21"/>
+      <c r="AC41" s="21"/>
+      <c r="AD41" s="21"/>
+      <c r="AE41" s="21"/>
+      <c r="AF41" s="21"/>
+      <c r="AG41" s="21"/>
+      <c r="AH41" s="30"/>
     </row>
-    <row r="42" spans="1:43" ht="21.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="5" t="s">
         <v>73</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C42" s="5">
         <v>0</v>
@@ -4317,436 +4333,376 @@
       <c r="J42" s="6">
         <v>0</v>
       </c>
-      <c r="K42" s="23" t="s">
+      <c r="K42" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="L42" s="21"/>
+      <c r="M42" s="21"/>
+      <c r="N42" s="21"/>
+      <c r="O42" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="L42" s="28"/>
-      <c r="M42" s="28"/>
-      <c r="N42" s="28"/>
-      <c r="O42" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="P42" s="22"/>
-      <c r="Q42" s="22"/>
-      <c r="R42" s="23"/>
-      <c r="S42" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="T42" s="28"/>
-      <c r="U42" s="28"/>
-      <c r="V42" s="28"/>
-      <c r="W42" s="28"/>
-      <c r="X42" s="28"/>
-      <c r="Y42" s="28"/>
-      <c r="Z42" s="28"/>
-      <c r="AA42" s="28"/>
-      <c r="AB42" s="28"/>
-      <c r="AC42" s="28"/>
-      <c r="AD42" s="28"/>
-      <c r="AE42" s="28"/>
-      <c r="AF42" s="28"/>
-      <c r="AG42" s="28"/>
-      <c r="AH42" s="29"/>
+      <c r="P42" s="29"/>
+      <c r="Q42" s="29"/>
+      <c r="R42" s="20"/>
+      <c r="S42" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="T42" s="21"/>
+      <c r="U42" s="21"/>
+      <c r="V42" s="21"/>
+      <c r="W42" s="21"/>
+      <c r="X42" s="21"/>
+      <c r="Y42" s="21"/>
+      <c r="Z42" s="21"/>
+      <c r="AA42" s="21"/>
+      <c r="AB42" s="21"/>
+      <c r="AC42" s="21"/>
+      <c r="AD42" s="21"/>
+      <c r="AE42" s="21"/>
+      <c r="AF42" s="21"/>
+      <c r="AG42" s="21"/>
+      <c r="AH42" s="30"/>
     </row>
-    <row r="43" spans="1:43" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B43" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="C43" s="5">
+        <v>0</v>
+      </c>
+      <c r="D43" s="1">
+        <v>0</v>
+      </c>
+      <c r="E43" s="1">
+        <v>1</v>
+      </c>
+      <c r="F43" s="1">
+        <v>0</v>
+      </c>
+      <c r="G43" s="1">
+        <v>0</v>
+      </c>
+      <c r="H43" s="6">
+        <v>0</v>
+      </c>
+      <c r="I43" s="5">
+        <v>0</v>
+      </c>
+      <c r="J43" s="6">
+        <v>0</v>
+      </c>
+      <c r="K43" s="27"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
+      <c r="P43" s="22"/>
+      <c r="Q43" s="22"/>
+      <c r="R43" s="22"/>
+      <c r="S43" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="T43" s="21"/>
+      <c r="U43" s="21"/>
+      <c r="V43" s="21"/>
+      <c r="W43" s="21"/>
+      <c r="X43" s="21"/>
+      <c r="Y43" s="21"/>
+      <c r="Z43" s="21"/>
+      <c r="AA43" s="21"/>
+      <c r="AB43" s="21"/>
+      <c r="AC43" s="21"/>
+      <c r="AD43" s="21"/>
+      <c r="AE43" s="21"/>
+      <c r="AF43" s="21"/>
+      <c r="AG43" s="21"/>
+      <c r="AH43" s="30"/>
+    </row>
+    <row r="44" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C44" s="5">
+        <v>0</v>
+      </c>
+      <c r="D44" s="1">
+        <v>0</v>
+      </c>
+      <c r="E44" s="1">
+        <v>1</v>
+      </c>
+      <c r="F44" s="1">
+        <v>0</v>
+      </c>
+      <c r="G44" s="1">
+        <v>0</v>
+      </c>
+      <c r="H44" s="6">
+        <v>1</v>
+      </c>
+      <c r="I44" s="5">
+        <v>0</v>
+      </c>
+      <c r="J44" s="6">
+        <v>0</v>
+      </c>
+      <c r="K44" s="27">
+        <v>0</v>
+      </c>
+      <c r="L44" s="22"/>
+      <c r="M44" s="22"/>
+      <c r="N44" s="22"/>
+      <c r="O44" s="22"/>
+      <c r="P44" s="22"/>
+      <c r="Q44" s="22"/>
+      <c r="R44" s="22"/>
+      <c r="S44" s="22"/>
+      <c r="T44" s="22"/>
+      <c r="U44" s="22"/>
+      <c r="V44" s="22"/>
+      <c r="W44" s="22"/>
+      <c r="X44" s="22"/>
+      <c r="Y44" s="22"/>
+      <c r="Z44" s="22"/>
+      <c r="AA44" s="22"/>
+      <c r="AB44" s="22"/>
+      <c r="AC44" s="22"/>
+      <c r="AD44" s="22"/>
+      <c r="AE44" s="22"/>
+      <c r="AF44" s="22"/>
+      <c r="AG44" s="22"/>
+      <c r="AH44" s="23"/>
+    </row>
+    <row r="45" spans="1:43" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C43" s="5">
-        <v>0</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1</v>
-      </c>
-      <c r="E43" s="1">
-        <v>0</v>
-      </c>
-      <c r="F43" s="1">
-        <v>0</v>
-      </c>
-      <c r="G43" s="1">
-        <v>0</v>
-      </c>
-      <c r="H43" s="6">
-        <v>1</v>
-      </c>
-      <c r="I43" s="5">
-        <v>1</v>
-      </c>
-      <c r="J43" s="6">
-        <v>0</v>
-      </c>
-      <c r="K43" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="L43" s="28"/>
-      <c r="M43" s="28"/>
-      <c r="N43" s="28"/>
-      <c r="O43" s="19">
-        <v>1</v>
-      </c>
-      <c r="P43" s="19">
-        <v>1</v>
-      </c>
-      <c r="Q43" s="19">
-        <v>1</v>
-      </c>
-      <c r="R43" s="19">
-        <v>1</v>
-      </c>
-      <c r="S43" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="T43" s="28"/>
-      <c r="U43" s="28"/>
-      <c r="V43" s="28"/>
-      <c r="W43" s="28"/>
-      <c r="X43" s="28"/>
-      <c r="Y43" s="28"/>
-      <c r="Z43" s="28"/>
-      <c r="AA43" s="28"/>
-      <c r="AB43" s="28"/>
-      <c r="AC43" s="28"/>
-      <c r="AD43" s="28"/>
-      <c r="AE43" s="28"/>
-      <c r="AF43" s="28"/>
-      <c r="AG43" s="28"/>
-      <c r="AH43" s="29"/>
+      <c r="B45" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C45" s="5">
+        <v>0</v>
+      </c>
+      <c r="D45" s="1">
+        <v>0</v>
+      </c>
+      <c r="E45" s="1">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1">
+        <v>0</v>
+      </c>
+      <c r="G45" s="1">
+        <v>1</v>
+      </c>
+      <c r="H45" s="6">
+        <v>0</v>
+      </c>
+      <c r="I45" s="5">
+        <v>0</v>
+      </c>
+      <c r="J45" s="6">
+        <v>0</v>
+      </c>
+      <c r="K45" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="L45" s="21"/>
+      <c r="M45" s="21"/>
+      <c r="N45" s="21"/>
+      <c r="O45" s="22">
+        <v>0</v>
+      </c>
+      <c r="P45" s="22"/>
+      <c r="Q45" s="22"/>
+      <c r="R45" s="22"/>
+      <c r="S45" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="T45" s="21"/>
+      <c r="U45" s="21"/>
+      <c r="V45" s="21"/>
+      <c r="W45" s="21"/>
+      <c r="X45" s="21"/>
+      <c r="Y45" s="21"/>
+      <c r="Z45" s="21"/>
+      <c r="AA45" s="21"/>
+      <c r="AB45" s="21"/>
+      <c r="AC45" s="21"/>
+      <c r="AD45" s="21"/>
+      <c r="AE45" s="21"/>
+      <c r="AF45" s="21"/>
+      <c r="AG45" s="21"/>
+      <c r="AH45" s="30"/>
     </row>
-    <row r="44" spans="1:43" ht="38.4" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B44" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C44" s="5">
-        <v>1</v>
-      </c>
-      <c r="D44" s="1">
-        <v>1</v>
-      </c>
-      <c r="E44" s="1">
-        <v>1</v>
-      </c>
-      <c r="F44" s="1">
-        <v>0</v>
-      </c>
-      <c r="G44" s="1">
-        <v>0</v>
-      </c>
-      <c r="H44" s="6">
-        <v>1</v>
-      </c>
-      <c r="I44" s="5">
-        <v>1</v>
-      </c>
-      <c r="J44" s="6">
-        <v>0</v>
-      </c>
-      <c r="K44" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="L44" s="28"/>
-      <c r="M44" s="28"/>
-      <c r="N44" s="28"/>
-      <c r="O44" s="19">
-        <v>1</v>
-      </c>
-      <c r="P44" s="19">
-        <v>1</v>
-      </c>
-      <c r="Q44" s="19">
-        <v>1</v>
-      </c>
-      <c r="R44" s="19">
-        <v>1</v>
-      </c>
-      <c r="S44" s="28" t="s">
-        <v>126</v>
-      </c>
-      <c r="T44" s="28"/>
-      <c r="U44" s="28"/>
-      <c r="V44" s="28"/>
-      <c r="W44" s="28"/>
-      <c r="X44" s="28"/>
-      <c r="Y44" s="28"/>
-      <c r="Z44" s="28"/>
-      <c r="AA44" s="28"/>
-      <c r="AB44" s="28"/>
-      <c r="AC44" s="28"/>
-      <c r="AD44" s="28"/>
-      <c r="AE44" s="28"/>
-      <c r="AF44" s="28"/>
-      <c r="AG44" s="28"/>
-      <c r="AH44" s="29"/>
-    </row>
-    <row r="45" spans="1:43" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B45" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="C45" s="5">
-        <v>0</v>
-      </c>
-      <c r="D45" s="1">
-        <v>0</v>
-      </c>
-      <c r="E45" s="1">
-        <v>1</v>
-      </c>
-      <c r="F45" s="1">
-        <v>0</v>
-      </c>
-      <c r="G45" s="1">
-        <v>0</v>
-      </c>
-      <c r="H45" s="6">
-        <v>0</v>
-      </c>
-      <c r="I45" s="5">
-        <v>0</v>
-      </c>
-      <c r="J45" s="6">
-        <v>0</v>
-      </c>
-      <c r="K45" s="27"/>
-      <c r="L45" s="33"/>
-      <c r="M45" s="33"/>
-      <c r="N45" s="33"/>
-      <c r="O45" s="33"/>
-      <c r="P45" s="33"/>
-      <c r="Q45" s="33"/>
-      <c r="R45" s="33"/>
-      <c r="S45" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="T45" s="28"/>
-      <c r="U45" s="28"/>
-      <c r="V45" s="28"/>
-      <c r="W45" s="28"/>
-      <c r="X45" s="28"/>
-      <c r="Y45" s="28"/>
-      <c r="Z45" s="28"/>
-      <c r="AA45" s="28"/>
-      <c r="AB45" s="28"/>
-      <c r="AC45" s="28"/>
-      <c r="AD45" s="28"/>
-      <c r="AE45" s="28"/>
-      <c r="AF45" s="28"/>
-      <c r="AG45" s="28"/>
-      <c r="AH45" s="29"/>
-    </row>
-    <row r="46" spans="1:43" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B46" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="C46" s="5">
-        <v>0</v>
-      </c>
-      <c r="D46" s="1">
-        <v>0</v>
-      </c>
-      <c r="E46" s="1">
-        <v>1</v>
-      </c>
-      <c r="F46" s="1">
-        <v>0</v>
-      </c>
-      <c r="G46" s="1">
-        <v>0</v>
-      </c>
-      <c r="H46" s="6">
-        <v>1</v>
-      </c>
-      <c r="I46" s="5">
-        <v>0</v>
-      </c>
-      <c r="J46" s="6">
-        <v>0</v>
-      </c>
-      <c r="K46" s="27">
-        <v>0</v>
-      </c>
-      <c r="L46" s="33"/>
-      <c r="M46" s="33"/>
-      <c r="N46" s="33"/>
-      <c r="O46" s="33"/>
-      <c r="P46" s="33"/>
-      <c r="Q46" s="33"/>
-      <c r="R46" s="33"/>
-      <c r="S46" s="33"/>
-      <c r="T46" s="33"/>
-      <c r="U46" s="33"/>
-      <c r="V46" s="33"/>
-      <c r="W46" s="33"/>
-      <c r="X46" s="33"/>
-      <c r="Y46" s="33"/>
-      <c r="Z46" s="33"/>
-      <c r="AA46" s="33"/>
-      <c r="AB46" s="33"/>
-      <c r="AC46" s="33"/>
-      <c r="AD46" s="33"/>
-      <c r="AE46" s="33"/>
-      <c r="AF46" s="33"/>
-      <c r="AG46" s="33"/>
-      <c r="AH46" s="34"/>
-    </row>
-    <row r="47" spans="1:43" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" s="5">
-        <v>0</v>
-      </c>
-      <c r="D47" s="1">
-        <v>0</v>
-      </c>
-      <c r="E47" s="1">
-        <v>1</v>
-      </c>
-      <c r="F47" s="1">
-        <v>0</v>
-      </c>
-      <c r="G47" s="1">
-        <v>1</v>
-      </c>
-      <c r="H47" s="6">
-        <v>0</v>
-      </c>
-      <c r="I47" s="5">
-        <v>0</v>
-      </c>
-      <c r="J47" s="6">
-        <v>0</v>
-      </c>
-      <c r="K47" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="L47" s="28"/>
-      <c r="M47" s="28"/>
-      <c r="N47" s="28"/>
-      <c r="O47" s="33">
-        <v>0</v>
-      </c>
-      <c r="P47" s="33"/>
-      <c r="Q47" s="33"/>
-      <c r="R47" s="33"/>
-      <c r="S47" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="T47" s="28"/>
-      <c r="U47" s="28"/>
-      <c r="V47" s="28"/>
-      <c r="W47" s="28"/>
-      <c r="X47" s="28"/>
-      <c r="Y47" s="28"/>
-      <c r="Z47" s="28"/>
-      <c r="AA47" s="28"/>
-      <c r="AB47" s="28"/>
-      <c r="AC47" s="28"/>
-      <c r="AD47" s="28"/>
-      <c r="AE47" s="28"/>
-      <c r="AF47" s="28"/>
-      <c r="AG47" s="28"/>
-      <c r="AH47" s="29"/>
-    </row>
-    <row r="48" spans="1:43" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C48" s="7">
-        <v>0</v>
-      </c>
-      <c r="D48" s="9">
-        <v>0</v>
-      </c>
-      <c r="E48" s="9">
-        <v>1</v>
-      </c>
-      <c r="F48" s="9">
-        <v>1</v>
-      </c>
-      <c r="G48" s="9">
-        <v>1</v>
-      </c>
-      <c r="H48" s="8">
-        <v>1</v>
-      </c>
-      <c r="I48" s="7">
-        <v>0</v>
-      </c>
-      <c r="J48" s="8">
-        <v>0</v>
-      </c>
-      <c r="K48" s="30">
-        <v>0</v>
-      </c>
-      <c r="L48" s="31"/>
-      <c r="M48" s="31"/>
-      <c r="N48" s="31"/>
-      <c r="O48" s="31"/>
-      <c r="P48" s="31"/>
-      <c r="Q48" s="31"/>
-      <c r="R48" s="31"/>
-      <c r="S48" s="31"/>
-      <c r="T48" s="31"/>
-      <c r="U48" s="31"/>
-      <c r="V48" s="31"/>
-      <c r="W48" s="31"/>
-      <c r="X48" s="31"/>
-      <c r="Y48" s="31"/>
-      <c r="Z48" s="31"/>
-      <c r="AA48" s="31"/>
-      <c r="AB48" s="31"/>
-      <c r="AC48" s="31"/>
-      <c r="AD48" s="31"/>
-      <c r="AE48" s="31"/>
-      <c r="AF48" s="31"/>
-      <c r="AG48" s="31"/>
-      <c r="AH48" s="32"/>
+    <row r="46" spans="1:43" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A46" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C46" s="7">
+        <v>0</v>
+      </c>
+      <c r="D46" s="9">
+        <v>0</v>
+      </c>
+      <c r="E46" s="9">
+        <v>1</v>
+      </c>
+      <c r="F46" s="9">
+        <v>1</v>
+      </c>
+      <c r="G46" s="9">
+        <v>1</v>
+      </c>
+      <c r="H46" s="8">
+        <v>1</v>
+      </c>
+      <c r="I46" s="7">
+        <v>0</v>
+      </c>
+      <c r="J46" s="8">
+        <v>0</v>
+      </c>
+      <c r="K46" s="42">
+        <v>0</v>
+      </c>
+      <c r="L46" s="43"/>
+      <c r="M46" s="43"/>
+      <c r="N46" s="43"/>
+      <c r="O46" s="43"/>
+      <c r="P46" s="43"/>
+      <c r="Q46" s="43"/>
+      <c r="R46" s="43"/>
+      <c r="S46" s="43"/>
+      <c r="T46" s="43"/>
+      <c r="U46" s="43"/>
+      <c r="V46" s="43"/>
+      <c r="W46" s="43"/>
+      <c r="X46" s="43"/>
+      <c r="Y46" s="43"/>
+      <c r="Z46" s="43"/>
+      <c r="AA46" s="43"/>
+      <c r="AB46" s="43"/>
+      <c r="AC46" s="43"/>
+      <c r="AD46" s="43"/>
+      <c r="AE46" s="43"/>
+      <c r="AF46" s="43"/>
+      <c r="AG46" s="43"/>
+      <c r="AH46" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="154">
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="O26:R26"/>
-    <mergeCell ref="S26:V26"/>
-    <mergeCell ref="W26:AH26"/>
-    <mergeCell ref="S31:V31"/>
-    <mergeCell ref="S32:V32"/>
-    <mergeCell ref="W31:AH31"/>
-    <mergeCell ref="W32:AH32"/>
-    <mergeCell ref="S33:AH33"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="O31:R31"/>
-    <mergeCell ref="O32:R32"/>
-    <mergeCell ref="O33:R33"/>
-    <mergeCell ref="K24:N24"/>
-    <mergeCell ref="O24:R24"/>
-    <mergeCell ref="S24:V24"/>
-    <mergeCell ref="W24:AH24"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="O25:R25"/>
-    <mergeCell ref="S25:V25"/>
-    <mergeCell ref="W25:AH25"/>
-    <mergeCell ref="S23:AD23"/>
-    <mergeCell ref="AE23:AH23"/>
+  <mergeCells count="150">
+    <mergeCell ref="K40:N40"/>
+    <mergeCell ref="O40:AH40"/>
+    <mergeCell ref="O36:R36"/>
+    <mergeCell ref="S36:AH36"/>
+    <mergeCell ref="O37:R37"/>
+    <mergeCell ref="S37:AH37"/>
+    <mergeCell ref="O38:R38"/>
+    <mergeCell ref="S38:AH38"/>
+    <mergeCell ref="O39:R39"/>
+    <mergeCell ref="S39:AH39"/>
+    <mergeCell ref="K36:N36"/>
+    <mergeCell ref="K37:N37"/>
+    <mergeCell ref="K38:N38"/>
+    <mergeCell ref="K39:N39"/>
+    <mergeCell ref="K46:AH46"/>
+    <mergeCell ref="S45:AH45"/>
+    <mergeCell ref="O45:R45"/>
+    <mergeCell ref="K45:N45"/>
+    <mergeCell ref="S43:AH43"/>
+    <mergeCell ref="K43:R43"/>
+    <mergeCell ref="K44:AH44"/>
+    <mergeCell ref="A1:AL1"/>
+    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="O27:R27"/>
+    <mergeCell ref="S27:V27"/>
+    <mergeCell ref="W27:AH27"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="O28:R28"/>
+    <mergeCell ref="S28:V28"/>
+    <mergeCell ref="W28:AH28"/>
+    <mergeCell ref="K29:N29"/>
+    <mergeCell ref="O29:R29"/>
+    <mergeCell ref="S29:AH29"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="O30:R30"/>
+    <mergeCell ref="S30:AH30"/>
+    <mergeCell ref="K34:N34"/>
+    <mergeCell ref="K35:N35"/>
+    <mergeCell ref="S41:AH41"/>
+    <mergeCell ref="S42:AH42"/>
+    <mergeCell ref="K42:N42"/>
+    <mergeCell ref="K41:N41"/>
+    <mergeCell ref="O41:R41"/>
+    <mergeCell ref="O42:R42"/>
+    <mergeCell ref="O34:R34"/>
+    <mergeCell ref="S34:AH34"/>
+    <mergeCell ref="O35:R35"/>
+    <mergeCell ref="S35:AH35"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="S5:V5"/>
+    <mergeCell ref="W5:AH5"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="S9:V9"/>
+    <mergeCell ref="W9:AH9"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="S10:V10"/>
+    <mergeCell ref="W10:AH10"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="W6:AH6"/>
+    <mergeCell ref="S8:V8"/>
+    <mergeCell ref="W8:AH8"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="S7:V7"/>
+    <mergeCell ref="W7:AH7"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="K2:R2"/>
+    <mergeCell ref="S2:Z2"/>
+    <mergeCell ref="AA2:AH2"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="K3:AH3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K4:AH4"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="O8:R8"/>
+    <mergeCell ref="K15:N15"/>
+    <mergeCell ref="O15:R15"/>
+    <mergeCell ref="S15:AH15"/>
+    <mergeCell ref="K16:N16"/>
+    <mergeCell ref="O16:R16"/>
+    <mergeCell ref="S16:AH16"/>
+    <mergeCell ref="AL2:AL3"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="K13:N13"/>
+    <mergeCell ref="O13:R13"/>
+    <mergeCell ref="S13:AH13"/>
+    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="O14:R14"/>
+    <mergeCell ref="S14:AH14"/>
+    <mergeCell ref="K11:N11"/>
+    <mergeCell ref="O11:R11"/>
+    <mergeCell ref="S11:V11"/>
+    <mergeCell ref="W11:AH11"/>
+    <mergeCell ref="K12:N12"/>
+    <mergeCell ref="O12:R12"/>
+    <mergeCell ref="S12:V12"/>
+    <mergeCell ref="W12:AH12"/>
     <mergeCell ref="K9:N9"/>
     <mergeCell ref="O9:R9"/>
     <mergeCell ref="K22:N22"/>
@@ -4771,111 +4727,31 @@
     <mergeCell ref="K18:N18"/>
     <mergeCell ref="O18:R18"/>
     <mergeCell ref="S18:AH18"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="O8:R8"/>
-    <mergeCell ref="K15:N15"/>
-    <mergeCell ref="O15:R15"/>
-    <mergeCell ref="S15:AH15"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="O16:R16"/>
-    <mergeCell ref="S16:AH16"/>
-    <mergeCell ref="AL2:AL3"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="K13:N13"/>
-    <mergeCell ref="O13:R13"/>
-    <mergeCell ref="S13:AH13"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="O14:R14"/>
-    <mergeCell ref="S14:AH14"/>
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="O11:R11"/>
-    <mergeCell ref="S11:V11"/>
-    <mergeCell ref="W11:AH11"/>
-    <mergeCell ref="K12:N12"/>
-    <mergeCell ref="O12:R12"/>
-    <mergeCell ref="S12:V12"/>
-    <mergeCell ref="W12:AH12"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="K2:R2"/>
-    <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AH2"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="K3:AH3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K4:AH4"/>
-    <mergeCell ref="O34:R34"/>
-    <mergeCell ref="S34:AH34"/>
-    <mergeCell ref="O35:R35"/>
-    <mergeCell ref="S35:AH35"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="O5:R5"/>
-    <mergeCell ref="S5:V5"/>
-    <mergeCell ref="W5:AH5"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="S9:V9"/>
-    <mergeCell ref="W9:AH9"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="O10:R10"/>
-    <mergeCell ref="S10:V10"/>
-    <mergeCell ref="W10:AH10"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="W6:AH6"/>
-    <mergeCell ref="S8:V8"/>
-    <mergeCell ref="W8:AH8"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="S7:V7"/>
-    <mergeCell ref="W7:AH7"/>
-    <mergeCell ref="S44:AH44"/>
-    <mergeCell ref="S41:AH41"/>
-    <mergeCell ref="S42:AH42"/>
-    <mergeCell ref="S43:AH43"/>
-    <mergeCell ref="K43:N43"/>
-    <mergeCell ref="K44:N44"/>
-    <mergeCell ref="K42:N42"/>
-    <mergeCell ref="K41:N41"/>
-    <mergeCell ref="O41:R41"/>
-    <mergeCell ref="O42:R42"/>
-    <mergeCell ref="K48:AH48"/>
-    <mergeCell ref="S47:AH47"/>
-    <mergeCell ref="O47:R47"/>
-    <mergeCell ref="K47:N47"/>
-    <mergeCell ref="S45:AH45"/>
-    <mergeCell ref="K45:R45"/>
-    <mergeCell ref="K46:AH46"/>
-    <mergeCell ref="A1:AL1"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="O27:R27"/>
-    <mergeCell ref="S27:V27"/>
-    <mergeCell ref="W27:AH27"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="O28:R28"/>
-    <mergeCell ref="S28:V28"/>
-    <mergeCell ref="W28:AH28"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="O29:R29"/>
-    <mergeCell ref="S29:AH29"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="O30:R30"/>
-    <mergeCell ref="S30:AH30"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="K35:N35"/>
-    <mergeCell ref="K40:N40"/>
-    <mergeCell ref="O40:AH40"/>
-    <mergeCell ref="O36:R36"/>
-    <mergeCell ref="S36:AH36"/>
-    <mergeCell ref="O37:R37"/>
-    <mergeCell ref="S37:AH37"/>
-    <mergeCell ref="O38:R38"/>
-    <mergeCell ref="S38:AH38"/>
-    <mergeCell ref="O39:R39"/>
-    <mergeCell ref="S39:AH39"/>
-    <mergeCell ref="K36:N36"/>
-    <mergeCell ref="K37:N37"/>
-    <mergeCell ref="K38:N38"/>
-    <mergeCell ref="K39:N39"/>
+    <mergeCell ref="K24:N24"/>
+    <mergeCell ref="O24:R24"/>
+    <mergeCell ref="S24:V24"/>
+    <mergeCell ref="W24:AH24"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="O25:R25"/>
+    <mergeCell ref="S25:V25"/>
+    <mergeCell ref="W25:AH25"/>
+    <mergeCell ref="S23:AD23"/>
+    <mergeCell ref="AE23:AH23"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="O26:R26"/>
+    <mergeCell ref="S26:V26"/>
+    <mergeCell ref="W26:AH26"/>
+    <mergeCell ref="S31:V31"/>
+    <mergeCell ref="S32:V32"/>
+    <mergeCell ref="W31:AH31"/>
+    <mergeCell ref="W32:AH32"/>
+    <mergeCell ref="S33:AH33"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="K32:N32"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="O31:R31"/>
+    <mergeCell ref="O32:R32"/>
+    <mergeCell ref="O33:R33"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C2:J2 C3:I3 C4:J1048576">

</xml_diff>